<commit_message>
New test_hand and FSR
</commit_message>
<xml_diff>
--- a/data/FSR.xlsx
+++ b/data/FSR.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/1a5740ffd8a34622/Escritorio/preprosthetic-robotic-hand/experimental_data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/1a5740ffd8a34622/Documentos/GitHub/preprosthetic-robotic-hand/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="30" documentId="8_{02DA831A-85AE-4687-ACCE-21D19AE54C97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{80417496-79C9-412E-98E2-303A4F870092}"/>
+  <xr:revisionPtr revIDLastSave="31" documentId="8_{02DA831A-85AE-4687-ACCE-21D19AE54C97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6233EC25-C21E-40AD-953E-D53301ABEB0B}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{F79691EB-FCD4-4BA8-B80D-061A19F0D7E1}"/>
+    <workbookView xWindow="345" yWindow="345" windowWidth="15375" windowHeight="7785" xr2:uid="{F79691EB-FCD4-4BA8-B80D-061A19F0D7E1}"/>
   </bookViews>
   <sheets>
     <sheet name="Data" sheetId="1" r:id="rId1"/>
@@ -36,48 +36,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="6">
   <si>
     <t>10k</t>
   </si>
   <si>
     <t>1k</t>
-  </si>
-  <si>
-    <t>TB6612FNG</t>
-  </si>
-  <si>
-    <t>A</t>
-  </si>
-  <si>
-    <t>mA</t>
-  </si>
-  <si>
-    <t>Encoder negativo</t>
-  </si>
-  <si>
-    <t>Fuente</t>
-  </si>
-  <si>
-    <t>Encoder positivo</t>
-  </si>
-  <si>
-    <t>fuente</t>
-  </si>
-  <si>
-    <t>Salida</t>
-  </si>
-  <si>
-    <t>Tornillo M3</t>
-  </si>
-  <si>
-    <t>Cant</t>
-  </si>
-  <si>
-    <t>esquinero</t>
-  </si>
-  <si>
-    <t>doble</t>
   </si>
   <si>
     <t>Force (N)</t>
@@ -146,12 +110,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -494,7 +457,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B31C556F-2490-4AF3-811A-04DB6AC5612C}">
-  <dimension ref="B2:I61"/>
+  <dimension ref="B2:E10"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="16.85546875" bestFit="1" customWidth="1"/>
@@ -505,13 +468,13 @@
     <col min="13" max="14" width="15.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="D2" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="E2" s="4"/>
-    </row>
-    <row r="3" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="D2" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="E2" s="3"/>
+    </row>
+    <row r="3" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
       <c r="D3" s="1" t="s">
@@ -521,25 +484,21 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B4" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="F4" s="2"/>
-      <c r="G4" s="2"/>
-      <c r="H4" s="2"/>
-      <c r="I4" s="2"/>
-    </row>
-    <row r="5" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B4" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B5" s="1">
         <v>130</v>
       </c>
@@ -553,17 +512,13 @@
       <c r="E5" s="1">
         <v>1320</v>
       </c>
-      <c r="F5" s="2"/>
-      <c r="G5" s="2"/>
-      <c r="H5" s="2"/>
-      <c r="I5" s="2"/>
-    </row>
-    <row r="6" spans="2:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="6" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B6" s="1">
         <v>140</v>
       </c>
       <c r="C6" s="1">
-        <f t="shared" ref="C6:C10" si="0">B6*(9.81/1000)</f>
+        <f t="shared" ref="C6:C9" si="0">B6*(9.81/1000)</f>
         <v>1.3734000000000002</v>
       </c>
       <c r="D6" s="1">
@@ -572,12 +527,8 @@
       <c r="E6" s="1">
         <v>1420</v>
       </c>
-      <c r="F6" s="2"/>
-      <c r="G6" s="2"/>
-      <c r="H6" s="2"/>
-      <c r="I6" s="2"/>
-    </row>
-    <row r="7" spans="2:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="7" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B7" s="1">
         <v>150</v>
       </c>
@@ -591,12 +542,8 @@
       <c r="E7" s="1">
         <v>1480</v>
       </c>
-      <c r="F7" s="2"/>
-      <c r="G7" s="2"/>
-      <c r="H7" s="2"/>
-      <c r="I7" s="2"/>
-    </row>
-    <row r="8" spans="2:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="8" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B8" s="1">
         <v>170</v>
       </c>
@@ -610,12 +557,8 @@
       <c r="E8" s="1">
         <v>1540</v>
       </c>
-      <c r="F8" s="2"/>
-      <c r="G8" s="2"/>
-      <c r="H8" s="2"/>
-      <c r="I8" s="2"/>
-    </row>
-    <row r="9" spans="2:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="9" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B9" s="1">
         <v>180</v>
       </c>
@@ -629,12 +572,8 @@
       <c r="E9" s="1">
         <v>1580</v>
       </c>
-      <c r="F9" s="2"/>
-      <c r="G9" s="2"/>
-      <c r="H9" s="2"/>
-      <c r="I9" s="2"/>
-    </row>
-    <row r="10" spans="2:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="10" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B10" s="1">
         <v>230</v>
       </c>
@@ -647,121 +586,6 @@
       </c>
       <c r="E10" s="1">
         <v>1900</v>
-      </c>
-      <c r="F10" s="2"/>
-      <c r="G10" s="2"/>
-      <c r="H10" s="2"/>
-      <c r="I10" s="2"/>
-    </row>
-    <row r="15" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="E15" s="2"/>
-      <c r="F15" s="2"/>
-    </row>
-    <row r="16" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="E16" s="2"/>
-      <c r="F16" s="2"/>
-    </row>
-    <row r="17" spans="5:6" x14ac:dyDescent="0.25">
-      <c r="E17" s="2"/>
-      <c r="F17" s="2"/>
-    </row>
-    <row r="18" spans="5:6" x14ac:dyDescent="0.25">
-      <c r="E18" s="2"/>
-      <c r="F18" s="2"/>
-    </row>
-    <row r="19" spans="5:6" x14ac:dyDescent="0.25">
-      <c r="E19" s="2"/>
-      <c r="F19" s="2"/>
-    </row>
-    <row r="48" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C48" t="s">
-        <v>3</v>
-      </c>
-      <c r="D48" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="50" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C50">
-        <v>11</v>
-      </c>
-      <c r="D50" t="s">
-        <v>5</v>
-      </c>
-      <c r="E50">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="51" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C51">
-        <v>2</v>
-      </c>
-      <c r="D51" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="53" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C53">
-        <v>11</v>
-      </c>
-      <c r="D53" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="54" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C54">
-        <v>2</v>
-      </c>
-      <c r="D54" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="55" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C55">
-        <v>1</v>
-      </c>
-      <c r="D55" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="56" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C56">
-        <v>1</v>
-      </c>
-      <c r="D56" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="58" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C58" t="s">
-        <v>10</v>
-      </c>
-      <c r="D58" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="59" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C59" t="s">
-        <v>12</v>
-      </c>
-      <c r="D59">
-        <f>6*3</f>
-        <v>18</v>
-      </c>
-    </row>
-    <row r="60" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C60" t="s">
-        <v>13</v>
-      </c>
-      <c r="D60">
-        <f>10*2</f>
-        <v>20</v>
-      </c>
-    </row>
-    <row r="61" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D61">
-        <f>SUM(D59:D60)</f>
-        <v>38</v>
       </c>
     </row>
   </sheetData>

</xml_diff>